<commit_message>
Bulk Import template: dropdown lists read the Lists sheet through INDIRECT (rows added by the flow shifted the plain references, so the Area/Category/Rack dropdowns came out empty)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flows/Bulk_Import_Template_Master.xlsx
+++ b/flows/Bulk_Import_Template_Master.xlsx
@@ -2970,16 +2970,16 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Area" error="This area is not in your business line. The app will mark the row red." type="list" errorStyle="warning">
-      <formula1>OFFSET(Lists!$A$3,0,0,MAX(1,COUNTA(Lists!$A$3:$A$500)),1)</formula1>
+      <formula1>OFFSET(INDIRECT("Lists!$A$3"),0,0,MAX(1,COUNTA(INDIRECT("Lists!$A$3:$A$500"))),1)</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Category" error="Use a category code from the Lists sheet (the name also works)." type="list" errorStyle="warning">
-      <formula1>OFFSET(Lists!$C$3,0,0,MAX(1,COUNTA(Lists!$C$3:$C$500)),1)</formula1>
+      <formula1>OFFSET(INDIRECT("Lists!$C$3"),0,0,MAX(1,COUNTA(INDIRECT("Lists!$C$3:$C$500"))),1)</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="UOM" error="UOM must be one of the values in the Lists sheet." type="list" errorStyle="warning">
-      <formula1>Lists!$F$3:$F$16</formula1>
+      <formula1>INDIRECT("Lists!$F$3:$F$16")</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rack" error="This rack is not in the area of this row (see the Lists sheet)." type="list" errorStyle="warning">
-      <formula1>OFFSET(Lists!$H$2,IFERROR(MATCH($A2,Lists!$I$3:$I$500,0),498),0,MAX(1,COUNTIF(Lists!$I$3:$I$500,$A2)),1)</formula1>
+      <formula1>OFFSET(INDIRECT("Lists!$H$2"),IFERROR(MATCH($A2,INDIRECT("Lists!$I$3:$I$500"),0),498),0,MAX(1,COUNTIF(INDIRECT("Lists!$I$3:$I$500"),$A2)),1)</formula1>
     </dataValidation>
     <dataValidation sqref="G2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Number" error="Enter a number of 0 or more." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Bulk Import template: Rack dropdown only lists the racks of the row's area; without an area it shows '(Select the Area first)', the cell is greyed out (red when filled anyway), and an input message explains it
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flows/Bulk_Import_Template_Master.xlsx
+++ b/flows/Bulk_Import_Template_Master.xlsx
@@ -119,6 +119,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="00C42B1C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FDE7E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F1F3F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -647,7 +666,7 @@
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Rack: opsional. Dropdown hanya menampilkan rak milik Area di baris itu (isi Area dulu).</t>
+          <t>Rack: opsional. Dropdown hanya menampilkan rak milik Area di baris itu. Selama Area kosong, sel Rack abu-abu dan dropdown hanya berisi '(Select the Area first)'; sel jadi merah bila Rack diisi tanpa Area.</t>
         </is>
       </c>
     </row>
@@ -2968,6 +2987,14 @@
       <c r="I200" s="5" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="I2:I200">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND($A2="",$I2&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$A2=""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Area" error="This area is not in your business line. The app will mark the row red." type="list" errorStyle="warning">
       <formula1>OFFSET(INDIRECT("Lists!$A$3"),0,0,MAX(1,COUNTA(INDIRECT("Lists!$A$3:$A$500"))),1)</formula1>
@@ -2978,8 +3005,8 @@
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="UOM" error="UOM must be one of the values in the Lists sheet." type="list" errorStyle="warning">
       <formula1>INDIRECT("Lists!$F$3:$F$16")</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rack" error="This rack is not in the area of this row (see the Lists sheet)." type="list" errorStyle="warning">
-      <formula1>IF($A2="",OFFSET(INDIRECT("Lists!$H$3"),0,0,MAX(1,COUNTA(INDIRECT("Lists!$H$3:$H$500"))),1),OFFSET(INDIRECT("Lists!$H$2"),IFERROR(MATCH($A2,INDIRECT("Lists!$I$3:$I$500"),0),498),0,MAX(1,COUNTIF(INDIRECT("Lists!$I$3:$I$500"),$A2)),1))</formula1>
+    <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Rack" error="This rack is not in the area of this row (see the Lists sheet)." promptTitle="Rack" prompt="Select the Area of this row first. The list shows only the racks of that area. Leave empty for no rack." type="list" errorStyle="warning">
+      <formula1>IF($A2="",INDIRECT("Lists!$M$3"),IF(COUNTIF(INDIRECT("Lists!$I$3:$I$500"),$A2)=0,INDIRECT("Lists!$M$4"),OFFSET(INDIRECT("Lists!$H$2"),MATCH($A2,INDIRECT("Lists!$I$3:$I$500"),0),0,COUNTIF(INDIRECT("Lists!$I$3:$I$500"),$A2),1)))</formula1>
     </dataValidation>
     <dataValidation sqref="G2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Number" error="Enter a number of 0 or more." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
@@ -2998,7 +3025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3053,11 +3080,21 @@
           <t>EA</t>
         </is>
       </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>(Select the Area first)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="F4" s="9" t="inlineStr">
         <is>
           <t>M</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>(No rack in this area)</t>
         </is>
       </c>
     </row>

</xml_diff>